<commit_message>
task 097: Blind holes start at the last depth used, or 2 x D
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/libraries/AWB_Holes.xlsx
+++ b/libraries/AWB_Holes.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="187">
   <si>
     <t xml:space="preserve">AWB Hole Data</t>
   </si>
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Tabs</t>
   </si>
   <si>
-    <t xml:space="preserve">Settings: tap depth rule, drill extra depth, fit colours, default units.</t>
+    <t xml:space="preserve">Settings: tap depth rule, drill extra depth, blind hole depth, fit colours, default units.</t>
   </si>
   <si>
     <t xml:space="preserve">Clearance: bolt clearance hole diameters for Close, Normal and Loose fit.</t>
@@ -614,6 +614,12 @@
   </si>
   <si>
     <t xml:space="preserve">Flat bottom (end mill or flat-bottom drill). Angle left blank.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blind depth multiplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A new blind clearance or dowel hole starts at the last depth used; the first time, at this x nominal diameter.</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1336,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -1403,66 +1409,77 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>36</v>
+        <v>185</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>220</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>40</v>
-      </c>
-      <c r="G7" s="11"/>
+        <v>186</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>220</v>
+      </c>
+      <c r="E8" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="F8" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="E8" s="10" t="n">
-        <v>100</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>220</v>
-      </c>
-      <c r="G8" s="12"/>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>40</v>
       </c>
       <c r="E9" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>220</v>
+      </c>
+      <c r="G9" s="12"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" s="10" t="n">
         <v>170</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F10" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="G9" s="13"/>
+      <c r="G10" s="13"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
task 106: Dowel seats sized in the window
A dowel with a counterbore or countersink hides Fastener type and shows its
own seat boxes, starting from the last values used for that units and size,
then the Dowel tab's new seat columns, then the same-size seat row. The
counterbore depth takes expressions. Also commits the STATUS.md handoff.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/libraries/AWB_Holes.xlsx
+++ b/libraries/AWB_Holes.xlsx
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="188">
   <si>
     <t xml:space="preserve">AWB Hole Data</t>
   </si>
@@ -109,7 +109,7 @@
     <t xml:space="preserve">Tapped: tap drill per thread; default thread and drill depths are calculated from Settings and can be changed per hole in the window.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dowel: dowel and precision hole sizes.</t>
+    <t xml:space="preserve">Dowel: dowel and precision hole sizes. Cbore dia, Cbore depth, Csink dia and Csink angle are where the counterbore or countersink of a dowel hole starts; they follow no screw, and can be changed per hole in the window.</t>
   </si>
   <si>
     <t xml:space="preserve">Drill Point: bottom shapes for blind holes (118 deg, 90 deg, flat), and which one is the default.</t>
@@ -620,6 +620,9 @@
   </si>
   <si>
     <t xml:space="preserve">A new blind clearance or dowel hole starts at the last depth used; the first time, at this x nominal diameter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Csink angle</t>
   </si>
 </sst>
 </file>
@@ -3702,13 +3705,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3734,6 +3741,18 @@
       <c r="D4" s="15" t="s">
         <v>52</v>
       </c>
+      <c r="E4" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
@@ -3748,6 +3767,18 @@
       <c r="D5" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -3762,6 +3793,18 @@
       <c r="D6" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E6" s="16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
@@ -3776,6 +3819,18 @@
       <c r="D7" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E7" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
@@ -3790,6 +3845,18 @@
       <c r="D8" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
@@ -3804,6 +3871,18 @@
       <c r="D9" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E9" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
@@ -3818,6 +3897,18 @@
       <c r="D10" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E10" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
@@ -3832,6 +3923,18 @@
       <c r="D11" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E11" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
@@ -3846,6 +3949,18 @@
       <c r="D12" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E12" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
@@ -3860,6 +3975,18 @@
       <c r="D13" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E13" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
@@ -3873,6 +4000,18 @@
       </c>
       <c r="D14" s="10" t="s">
         <v>54</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3888,6 +4027,18 @@
       <c r="D15" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E15" s="16" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
@@ -3902,6 +4053,18 @@
       <c r="D16" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E16" s="16" t="n">
+        <v>0.2275</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>0.09375</v>
+      </c>
+      <c r="G16" s="16" t="n">
+        <v>0.2275</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
@@ -3916,6 +4079,18 @@
       <c r="D17" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E17" s="16" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="G17" s="16" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
@@ -3930,6 +4105,18 @@
       <c r="D18" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E18" s="16" t="n">
+        <v>0.3525</v>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>0.15625</v>
+      </c>
+      <c r="G18" s="16" t="n">
+        <v>0.3525</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
@@ -3944,6 +4131,18 @@
       <c r="D19" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="E19" s="16" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>0.1875</v>
+      </c>
+      <c r="G19" s="16" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
@@ -3957,6 +4156,18 @@
       </c>
       <c r="D20" s="10" t="s">
         <v>54</v>
+      </c>
+      <c r="E20" s="16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F20" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G20" s="16" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
task 111: hole workbook Spotface and Taper Tapped tabs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/libraries/AWB_Holes.xlsx
+++ b/libraries/AWB_Holes.xlsx
@@ -13,7 +13,9 @@
     <sheet name="Clearance" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Counterbore" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Countersink" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Spotface" sheetId="10" state="visible" r:id="rId13"/>
     <sheet name="Tapped" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Taper Tapped" sheetId="11" state="visible" r:id="rId14"/>
     <sheet name="Dowel" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Precision Tol" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Drill Point" sheetId="9" state="visible" r:id="rId11"/>
@@ -22,10 +24,12 @@
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Clearance!$A$4:$G$23</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Counterbore!$A$4:$G$21</definedName>
     <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Countersink!$A$4:$G$21</definedName>
-    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Dowel!$A$4:$D$20</definedName>
-    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'Drill Point'!$A$4:$E$7</definedName>
-    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Precision Tol'!$A$4:$I$12</definedName>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Tapped!$A$4:$I$26</definedName>
+    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">Dowel!$A$4:$D$20</definedName>
+    <definedName function="false" hidden="true" localSheetId="10" name="_xlnm._FilterDatabase" vbProcedure="false">'Drill Point'!$A$4:$E$7</definedName>
+    <definedName function="false" hidden="true" localSheetId="9" name="_xlnm._FilterDatabase" vbProcedure="false">'Precision Tol'!$A$4:$I$12</definedName>
+    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Tapped!$A$4:$I$26</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">Spotface!$A$4:$E$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Taper Tapped'!$A$4:$G$15</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -59,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="207">
   <si>
     <t xml:space="preserve">AWB Hole Data</t>
   </si>
@@ -623,6 +627,63 @@
   </si>
   <si>
     <t xml:space="preserve">Csink angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotfaces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A shallow flat seat for a bolt head or washer on a rough or sloping face. One row per hole size, matched by Size to the Clearance, Tapped and Dowel sizes. Starter values; check them. Spotface depth may be 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotface dia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotface depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taper tapped holes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tapered pipe threads. Thread type and Size must match Inventor's thread table (for example NPT 1/4, BSP Taper Internal Rc 1/4). Tap drill is for notes and hole tables; Inventor models its own. Default depths are calculated from Settings with the tap drill as D.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thread type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rc 1/8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSP Taper Internal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rc 1/4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rc 3/8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rc 1/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rc 3/4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotface: spotface diameter and depth per hole size; a spotface on a clearance, tapped or dowel hole of that size starts from them. Optional: a workbook without this tab still loads.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taper Tapped: tapered pipe threads (NPT, BSPT); Thread type and Size as Inventor's thread table names them. Tap drill is for notes and hole tables. Optional: a workbook without this tab still loads.</t>
   </si>
 </sst>
 </file>
@@ -1205,7 +1266,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -1297,33 +1358,743 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>15</v>
+        <v>205</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>17</v>
+        <v>206</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D16" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="D20" s="16" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D21" s="16" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:E21"/>
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A5:A304" type="list">
+      <formula1>"Metric,Imperial"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E304" type="list">
+      <formula1>"Y,N"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <f aca="false">ROUND(D5*Settings!$B$5,3)</f>
+        <v>12.6</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <f aca="false">ROUND(E5+D5*Settings!$B$6,3)</f>
+        <v>16.8</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <f aca="false">ROUND(D6*Settings!$B$5,3)</f>
+        <v>16.8</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <f aca="false">ROUND(E6+D6*Settings!$B$6,3)</f>
+        <v>22.4</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <f aca="false">ROUND(D7*Settings!$B$5,3)</f>
+        <v>22.2</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <f aca="false">ROUND(E7+D7*Settings!$B$6,3)</f>
+        <v>29.6</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <f aca="false">ROUND(D8*Settings!$B$5,3)</f>
+        <v>27.6</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <f aca="false">ROUND(E8+D8*Settings!$B$6,3)</f>
+        <v>36.8</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <f aca="false">ROUND(D9*Settings!$B$5,3)</f>
+        <v>36</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <f aca="false">ROUND(E9+D9*Settings!$B$6,3)</f>
+        <v>48</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <f aca="false">ROUND(D10*Settings!$B$5,3)</f>
+        <v>0.375</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <f aca="false">ROUND(E10+D10*Settings!$B$6,3)</f>
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <f aca="false">ROUND(D11*Settings!$B$5,3)</f>
+        <v>0.51</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <f aca="false">ROUND(E11+D11*Settings!$B$6,3)</f>
+        <v>0.68</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <f aca="false">ROUND(D12*Settings!$B$5,3)</f>
+        <v>0.66</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <f aca="false">ROUND(E12+D12*Settings!$B$6,3)</f>
+        <v>0.88</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <f aca="false">ROUND(D13*Settings!$B$5,3)</f>
+        <v>0.87</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <f aca="false">ROUND(E13+D13*Settings!$B$6,3)</f>
+        <v>1.16</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <f aca="false">ROUND(D14*Settings!$B$5,3)</f>
+        <v>1.08</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <f aca="false">ROUND(E14+D14*Settings!$B$6,3)</f>
+        <v>1.44</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <f aca="false">ROUND(D15*Settings!$B$5,3)</f>
+        <v>1.38</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <f aca="false">ROUND(E15+D15*Settings!$B$6,3)</f>
+        <v>1.84</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G15"/>
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="A5:A304" type="list">
+      <formula1>"Metric,Imperial"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G304" type="list">
+      <formula1>"Y,N"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>